<commit_message>
Reconcile weekly resource mappings
</commit_message>
<xml_diff>
--- a/Teacher Resources (Start Here)/06_STARLAB_Master_Print_Packet_Index.xlsx
+++ b/Teacher Resources (Start Here)/06_STARLAB_Master_Print_Packet_Index.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Re787411c930046a6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Packet Index" sheetId="2" r:id="R7978dcc6409c4216"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Print Queue" sheetId="3" r:id="R39178fa68a0e42ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Unit" sheetId="4" r:id="Ra2b73ef3b44745c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Type Key" sheetId="5" r:id="R194cf09786264db6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R34c44a9595d64e46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Packet Index" sheetId="2" r:id="R55b5b93884bc4974"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Print Queue" sheetId="3" r:id="R18f97d74571e4589"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Unit" sheetId="4" r:id="R4aeea3ddf42148e9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Type Key" sheetId="5" r:id="R664d5d85eaf247cc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -104,35 +104,15 @@
     <x:t xml:space="preserve">Deck 03</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Unit 2 / Week 4</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Unit 1; Unit 2</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Unit 1 Student Handout 4: Research Ethics and Integrity Agreement
-Unit 2 Student Handout 9: Safety and Risk Assessment
-Unit 2 Student Handout 10: Ethics and Approval Screening
-Unit 2 Appendix E: Risk Assessment Matrix
-Unit 2 Appendix F: Safety and Ethics Red Flags
-Unit 2 Appendix H: Project Approval Checklist</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Introduced early as course culture; revisited during formal project approval.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Experimental Design and Engineering Design Basics</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Deck 04</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Unit 2 / Week 3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Use first as a foundation lesson; revisit when students plan variables, criteria, and evidence.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Building a Formal Research Plan</x:t>
   </x:si>
   <x:si>
@@ -142,140 +122,34 @@
     <x:t xml:space="preserve">Unit 2</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Unit 2 Student Handout 1: Project Refinement Workshop
-Unit 2 Student Handout 2: Background Research Notes
-Unit 2 Student Handout 3: Hypothesis and Design Criteria Builder
-Unit 2 Student Handout 4: Variables, Controls, Criteria, and Constraints Organizer
-Unit 2 Student Handout 5: Evidence Planning Tool
-Unit 2 Student Handout 6: Materials and Equipment Planner
-Unit 2 Student Handout 7: Procedure and Testing Protocol Builder
-Unit 2 Student Handout 8: Data Collection Plan
-Unit 2 Student Handout 9: Safety and Risk Assessment
-Unit 2 Student Handout 10: Ethics and Approval Screening
-Unit 2 Student Handout 11: Project Timeline Planner
-Unit 2 Student Handout 12: Formal Research Plan Template
-Unit 2 Student Handout 13: Research Plan Conference Form
-Unit 2 Appendix H: Project Approval Checklist</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Project approval tracking sheet
-Mentor review template, if applicable</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">The main Unit 2 planning and approval deck.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Pilot Testing</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Deck 06</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Unit 3 / Week 5</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Unit 3</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Unit 3 Student Handout 1: Pilot Test Plan
-Unit 3 Student Handout 4: Pilot Test Reflection and Troubleshooting Log
-Unit 3 Student Handout 5: Method Revision Decision Chart
-Unit 3 Appendix A: What Is Pilot Testing?
-Unit 3 Appendix C: Safety Check Before Testing
-Unit 3 Appendix E: Troubleshooting Sentence Frames</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 Student Handout 3: Daily Research Journal Entry Template
-Unit 3 Appendix B: Research Journal Standards</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Launches the transition from planning to action.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Research Journals and Scientific Documentation</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Deck 07</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Unit 3 / Weeks 6–16</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 Student Handout 2: Research Journal Setup
-Unit 3 Student Handout 3: Daily Research Journal Entry Template
-Unit 3 Student Handout 4: Pilot Test Reflection and Troubleshooting Log
-Unit 3 Appendix B: Research Journal Standards</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 Student Handout 9: Weekly Progress Check-In
-Unit 3 Student Handout 19: Research Journal Self-Assessment
-Unit 3 Appendix Q: File and Data Organization Standards</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Introduce at journal setup; revisit throughout the long research phase.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Troubleshooting and Responsible Project Pivots</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Deck 08</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Unit 3 / Week 6</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 / Weeks 10, 13</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 Student Handout 4: Pilot Test Reflection and Troubleshooting Log
-Unit 3 Student Handout 5: Method Revision Decision Chart
-Unit 3 Student Handout 6: Revised Procedure Template
-Unit 3 Student Handout 11: Troubleshooting Conference Prep
-Unit 3 Student Handout 12: Mentor or Expert Feedback Log
-Unit 3 Appendix D: Types of Research Problems
-Unit 3 Appendix E: Troubleshooting Sentence Frames
-Unit 3 Appendix K: Responsible Project Pivots</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 Student Handout 9: Weekly Progress Check-In
-Unit 3 Student Handout 15: Post-Progress Report Action Plan
-Unit 3 Appendix P: Recovery Plan Options</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Use whenever a project stalls, pivots, or needs structured revision.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Data Organization: Raw Data vs. Clean Data</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Deck 09</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Unit 4 / Week 17</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 / Week 15–16 bridge</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Unit 3; Unit 4</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 4 Student Handout 1: Raw Data Inventory
-Unit 4 Student Handout 2: Clean Data Set Builder
-Unit 4 Student Handout 3: Data Cleaning Decision Log
-Unit 4 Student Handout 4: Week 17 Data Audit
-Unit 4 Appendix A: Raw Data vs. Clean Data
-Unit 4 Appendix B: Data Cleaning Rules
-Unit 4 Appendix C: Common Data Organization Problems</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 3 Student Handout 17: Data Audit and Organization Checklist
-Unit 3 Student Handout 18: Unit 3 Readiness for Analysis Review
-Unit 3 Appendix Q: File and Data Organization Standards
-Unit 3 Appendix R: Raw Data vs. Clean Data</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Primary Unit 4 launch deck; can be previewed near the end of Unit 3.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Choosing the Right Data Analysis Method</x:t>
@@ -470,12 +344,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Deck 19</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Unit 6 / Week 34</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Final course closure deck. No next deck after this.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Unit</x:t>
@@ -2020,7 +1888,7 @@
         <x:v>25</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="132" hidden="0" customHeight="1">
       <x:c r="A4" s="5">
         <x:v>3.0</x:v>
       </x:c>
@@ -2030,199 +1898,237 @@
       <x:c r="C4" s="5" t="s">
         <x:v>27</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="s">
-        <x:v>17</x:v>
-      </x:c>
-      <x:c r="E4" s="5" t="s">
+      <x:c r="D4" s="8" t="str">
+        <x:v>Unit 1 / Week 1</x:v>
+      </x:c>
+      <x:c r="E4" s="8" t="str">
+        <x:v>Unit 2 / Week 4</x:v>
+      </x:c>
+      <x:c r="F4" s="8" t="s">
         <x:v>28</x:v>
       </x:c>
-      <x:c r="F4" s="5" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="G4" s="5" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="H4" s="5" t="str">
-        <x:v>District-supplied safety, human-participant, privacy, media, fieldwork, equipment, chemical, drone, IRB/SRC, or other local forms as applicable</x:v>
-      </x:c>
-      <x:c r="I4" s="5" t="s">
-        <x:v>31</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
+      <x:c r="G4" s="8" t="str">
+        <x:v>Week 1 required:
+Unit 1 Student Handout 4: Research Ethics and Integrity Agreement
+Week 4 revisit required:
+Unit 2 Student Handout 9: Safety and Risk Assessment
+Unit 2 Student Handout 10: Ethics and Approval Screening
+Unit 2 Appendix E: Risk Assessment Matrix
+Unit 2 Appendix F: Safety and Ethics Red Flags
+Unit 2 Appendix H: Project Approval Checklist</x:v>
+      </x:c>
+      <x:c r="H4" s="8" t="str">
+        <x:v>District-supplied safety, human-participant, privacy, media, fieldwork, equipment, chemical, drone, IRB/SRC, or other local forms as applicable.</x:v>
+      </x:c>
+      <x:c r="I4" s="8" t="str">
+        <x:v>Introduce in Week 1 as course culture; revisit in Week 4 during formal project approval.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="145.1999969482422" hidden="0" customHeight="1">
       <x:c r="A5" s="5">
         <x:v>4.0</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>32</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>33</x:v>
-      </x:c>
-      <x:c r="D5" s="5" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="E5" s="5" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="F5" s="5" t="s">
-        <x:v>29</x:v>
-      </x:c>
-      <x:c r="G5" s="5" t="str">
-        <x:v>Unit 1 Student Handout 5: Experimental Design Practice
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="D5" s="8" t="str">
+        <x:v>Unit 1 / Week 2</x:v>
+      </x:c>
+      <x:c r="E5" s="8" t="str">
+        <x:v>Unit 2 / Week 3</x:v>
+      </x:c>
+      <x:c r="F5" s="8" t="s">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G5" s="8" t="str">
+        <x:v>Week 2 required:
+Unit 1 Student Handout 5: Experimental Design Practice
 Unit 1 Appendix D: Experimental Design Vocabulary
 Unit 1 Appendix G: Engineering Design Problem Guide
+Week 3 revisit required:
 Unit 2 Student Handout 3: Hypothesis and Design Criteria Builder
 Unit 2 Student Handout 4: Variables, Controls, Criteria, and Constraints Organizer
 Unit 2 Student Handout 5: Evidence Planning Tool</x:v>
       </x:c>
-      <x:c r="H5" s="5" t="str">
-        <x:v>Unit 1 Appendix I: Optional Project Card Sorting Activity
+      <x:c r="H5" s="8" t="str">
+        <x:v>Week 2 optional / teacher reference:
+Unit 1 Appendix I: Optional Project Card Sorting Activity
 Mini-investigation supplies</x:v>
       </x:c>
-      <x:c r="I5" s="5" t="s">
-        <x:v>35</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6">
+      <x:c r="I5" s="8" t="str">
+        <x:v>Use first as a Week 2 foundation lesson; revisit during Week 3 planning.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A6" s="5">
         <x:v>5.0</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>36</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>37</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="E6" s="5"/>
-      <x:c r="F6" s="5" t="s">
-        <x:v>38</x:v>
-      </x:c>
-      <x:c r="G6" s="5" t="s">
-        <x:v>39</x:v>
-      </x:c>
-      <x:c r="H6" s="5" t="s">
-        <x:v>40</x:v>
-      </x:c>
-      <x:c r="I6" s="5" t="s">
-        <x:v>41</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="D6" s="8" t="str">
+        <x:v>Unit 2 / Weeks 3-4</x:v>
+      </x:c>
+      <x:c r="E6" s="8" t="str"/>
+      <x:c r="F6" s="8" t="s">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="G6" s="8" t="str">
+        <x:v>Week 3 required:
+Unit 2 Student Handouts 1-5
+Unit 2 Appendices A-D
+Week 4 required:
+Unit 2 Student Handouts 6-13
+Unit 2 Appendices E-H</x:v>
+      </x:c>
+      <x:c r="H6" s="8" t="str">
+        <x:v>Week 4 optional / teacher reference:
+Unit 2 Appendix I: Mentor Feedback Request Template
+Unit 2 Appendix J: Sample Completed Planning Excerpt
+District-supplied approval and safety forms as applicable</x:v>
+      </x:c>
+      <x:c r="I6" s="8" t="str">
+        <x:v>The main Unit 2 planning and approval deck. The Week 3 and Week 4 packets are separated here to match the implementation calendar.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="39.599998474121094" hidden="0" customHeight="1">
       <x:c r="A7" s="5">
         <x:v>6.0</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>42</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C7" s="5" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="D7" s="5" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="E7" s="5"/>
-      <x:c r="F7" s="5" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G7" s="5" t="s">
-        <x:v>46</x:v>
-      </x:c>
-      <x:c r="H7" s="5" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="I7" s="5" t="s">
-        <x:v>48</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="D7" s="8" t="str">
+        <x:v>Unit 3 / Week 5</x:v>
+      </x:c>
+      <x:c r="E7" s="8" t="str"/>
+      <x:c r="F7" s="8" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="G7" s="8" t="str">
+        <x:v>Week 5 required weekly packet (shared with Deck 7):
+Unit 3 Student Handouts 1-3
+Unit 3 Appendices A-C</x:v>
+      </x:c>
+      <x:c r="H7" s="8" t="str"/>
+      <x:c r="I7" s="8" t="str">
+        <x:v>Launches pilot testing. Week 6 troubleshooting materials are introduced with Deck 8, not printed early with this deck.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A8" s="5">
         <x:v>7.0</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>49</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="C8" s="5" t="s">
-        <x:v>50</x:v>
-      </x:c>
-      <x:c r="D8" s="5" t="s">
-        <x:v>44</x:v>
-      </x:c>
-      <x:c r="E8" s="5" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F8" s="5" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G8" s="5" t="s">
-        <x:v>52</x:v>
-      </x:c>
-      <x:c r="H8" s="5" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="I8" s="5" t="s">
-        <x:v>54</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="9">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="D8" s="8" t="str">
+        <x:v>Unit 3 / Week 5</x:v>
+      </x:c>
+      <x:c r="E8" s="8" t="str">
+        <x:v>Unit 3 / Weeks 6-16 as needed</x:v>
+      </x:c>
+      <x:c r="F8" s="8" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="G8" s="8" t="str">
+        <x:v>Week 5 required weekly packet (shared with Deck 6):
+Unit 3 Student Handouts 1-3
+Unit 3 Appendices A-C</x:v>
+      </x:c>
+      <x:c r="H8" s="8" t="str">
+        <x:v>Later optional / teacher reference:
+Unit 3 Student Handout 9: Weekly Progress Check-In
+Unit 3 Student Handout 19: Research Journal Self-Assessment
+Unit 3 Appendix Q: File and Data Organization Standards</x:v>
+      </x:c>
+      <x:c r="I8" s="8" t="str">
+        <x:v>Introduce journal setup in Week 5; revisit documentation routines throughout Unit 3.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="79.19999694824219" hidden="0" customHeight="1">
       <x:c r="A9" s="5">
         <x:v>8.0</x:v>
       </x:c>
       <x:c r="B9" s="5" t="s">
-        <x:v>55</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="C9" s="5" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="D9" s="5" t="s">
-        <x:v>57</x:v>
-      </x:c>
-      <x:c r="E9" s="5" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="F9" s="5" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G9" s="5" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="H9" s="5" t="s">
-        <x:v>60</x:v>
-      </x:c>
-      <x:c r="I9" s="5" t="s">
-        <x:v>61</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="D9" s="8" t="str">
+        <x:v>Unit 3 / Week 6</x:v>
+      </x:c>
+      <x:c r="E9" s="8" t="str">
+        <x:v>Unit 3 / Weeks 7, 10, and 13 as needed</x:v>
+      </x:c>
+      <x:c r="F9" s="8" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="G9" s="8" t="str">
+        <x:v>Week 6 required:
+Unit 3 Student Handout 4: Pilot Test Reflection and Troubleshooting Log
+Unit 3 Student Handout 5: Method Revision Decision Chart
+Unit 3 Appendix D: Types of Research Problems
+Unit 3 Appendix E: Troubleshooting Sentence Frames</x:v>
+      </x:c>
+      <x:c r="H9" s="8" t="str">
+        <x:v>Week 7 revisit: Student Handouts 6-7; Appendices F-G
+Week 10 revisit: Student Handouts 11-12; Appendices K-L are optional / teacher reference
+Week 13 recovery use: Student Handout 15; Appendix P is optional / teacher reference</x:v>
+      </x:c>
+      <x:c r="I9" s="8" t="str">
+        <x:v>Use whenever a project stalls, pivots, or needs structured revision. Later-week resources remain in their assigned weekly packets.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="158.39999389648438" hidden="0" customHeight="1">
       <x:c r="A10" s="5">
         <x:v>9.0</x:v>
       </x:c>
       <x:c r="B10" s="5" t="s">
-        <x:v>62</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C10" s="5" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="D10" s="5" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="E10" s="5" t="s">
-        <x:v>65</x:v>
-      </x:c>
-      <x:c r="F10" s="5" t="s">
-        <x:v>66</x:v>
-      </x:c>
-      <x:c r="G10" s="5" t="s">
-        <x:v>67</x:v>
-      </x:c>
-      <x:c r="H10" s="5" t="s">
-        <x:v>68</x:v>
-      </x:c>
-      <x:c r="I10" s="5" t="s">
-        <x:v>69</x:v>
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="D10" s="8" t="str">
+        <x:v>Unit 3 / Week 15; Unit 4 / Week 17</x:v>
+      </x:c>
+      <x:c r="E10" s="8" t="str">
+        <x:v>Unit 3 / Week 16 revisit</x:v>
+      </x:c>
+      <x:c r="F10" s="8" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="G10" s="8" t="str">
+        <x:v>Week 15 required:
+Unit 3 Student Handout 17: Data Audit and Organization Checklist
+Unit 3 Appendices Q-R
+Week 16 required (Deck 9 revisit):
+Unit 3 Student Handout 18: Unit 3 Readiness for Analysis Review
+Unit 3 Student Handout 19: Research Journal Self-Assessment
+Week 17 required:
+Unit 4 Student Handouts 1-4
+Unit 4 Appendices A-C</x:v>
+      </x:c>
+      <x:c r="H10" s="8" t="str">
+        <x:v>Week 16 optional / teacher reference:
+Unit 3 Appendices S-U</x:v>
+      </x:c>
+      <x:c r="I10" s="8" t="str">
+        <x:v>Use as the Week 15 data-organization bridge, revisit in Week 16 for readiness, and teach again at the Unit 4 launch.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -2230,26 +2136,26 @@
         <x:v>10.0</x:v>
       </x:c>
       <x:c r="B11" s="5" t="s">
-        <x:v>70</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C11" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="D11" s="5" t="s">
-        <x:v>72</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="E11" s="5"/>
       <x:c r="F11" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="G11" s="5" t="s">
-        <x:v>74</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="H11" s="5" t="s">
-        <x:v>75</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="I11" s="5" t="s">
-        <x:v>76</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -2257,17 +2163,17 @@
         <x:v>11.0</x:v>
       </x:c>
       <x:c r="B12" s="5" t="s">
-        <x:v>77</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C12" s="5" t="s">
-        <x:v>78</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D12" s="5" t="s">
-        <x:v>79</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E12" s="5"/>
       <x:c r="F12" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="G12" s="5" t="str">
         <x:v>Unit 4 Student Handout 9: Graph and Visual Selection Tool
@@ -2277,10 +2183,10 @@
 Unit 4 Appendices H-K</x:v>
       </x:c>
       <x:c r="H12" s="5" t="s">
-        <x:v>80</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I12" s="5" t="s">
-        <x:v>81</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
@@ -2288,19 +2194,19 @@
         <x:v>12.0</x:v>
       </x:c>
       <x:c r="B13" s="5" t="s">
-        <x:v>82</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C13" s="5" t="s">
-        <x:v>83</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D13" s="5" t="s">
-        <x:v>79</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="E13" s="5" t="s">
-        <x:v>84</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="F13" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="G13" s="5" t="str">
         <x:v>Unit 4 Student Handout 11: Error, Uncertainty, and Limitations Review
@@ -2312,7 +2218,7 @@
 Project-specific uncertainty examples</x:v>
       </x:c>
       <x:c r="I13" s="5" t="s">
-        <x:v>85</x:v>
+        <x:v>59</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
@@ -2320,26 +2226,26 @@
         <x:v>13.0</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
-        <x:v>86</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C14" s="5" t="s">
-        <x:v>87</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="D14" s="5" t="s">
-        <x:v>88</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="E14" s="5"/>
       <x:c r="F14" s="5" t="s">
-        <x:v>89</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="G14" s="5" t="s">
-        <x:v>90</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="H14" s="5" t="s">
-        <x:v>91</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="I14" s="5" t="s">
-        <x:v>92</x:v>
+        <x:v>66</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
@@ -2347,28 +2253,28 @@
         <x:v>14.0</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
-        <x:v>93</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C15" s="5" t="s">
-        <x:v>94</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="D15" s="5" t="s">
-        <x:v>95</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="E15" s="5" t="s">
-        <x:v>96</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="F15" s="5" t="s">
-        <x:v>97</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="G15" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="H15" s="5" t="s">
-        <x:v>99</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="I15" s="5" t="s">
-        <x:v>100</x:v>
+        <x:v>74</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
@@ -2376,26 +2282,26 @@
         <x:v>15.0</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
-        <x:v>101</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="C16" s="5" t="s">
-        <x:v>102</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="D16" s="5" t="s">
-        <x:v>103</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="E16" s="5"/>
       <x:c r="F16" s="5" t="s">
-        <x:v>89</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="G16" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="H16" s="5" t="s">
-        <x:v>105</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="I16" s="5" t="s">
-        <x:v>106</x:v>
+        <x:v>80</x:v>
       </x:c>
     </x:row>
     <x:row r="17">
@@ -2403,19 +2309,19 @@
         <x:v>16.0</x:v>
       </x:c>
       <x:c r="B17" s="5" t="s">
-        <x:v>107</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="C17" s="5" t="s">
-        <x:v>108</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D17" s="5" t="s">
-        <x:v>109</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="E17" s="5" t="s">
-        <x:v>110</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="F17" s="5" t="s">
-        <x:v>111</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="G17" s="5" t="str">
         <x:v>Unit 5 Student Handout 10: Presentation Planning Guide
@@ -2428,7 +2334,7 @@
 Unit 6 Appendices I-K (teacher event references)</x:v>
       </x:c>
       <x:c r="I17" s="5" t="s">
-        <x:v>112</x:v>
+        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="18">
@@ -2436,19 +2342,19 @@
         <x:v>17.0</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
-        <x:v>113</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C18" s="5" t="s">
-        <x:v>114</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="D18" s="5" t="s">
-        <x:v>109</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="E18" s="5" t="s">
-        <x:v>115</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="F18" s="5" t="s">
-        <x:v>111</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="G18" s="5" t="str">
         <x:v>Unit 5 Student Handouts 10-11
@@ -2459,7 +2365,7 @@
         <x:v>Unit 6 Appendix L: final summative Oral Presentation rubric (teacher scoring reference)</x:v>
       </x:c>
       <x:c r="I18" s="5" t="s">
-        <x:v>116</x:v>
+        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
@@ -2467,56 +2373,56 @@
         <x:v>18.0</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
-        <x:v>117</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="C19" s="5" t="s">
-        <x:v>118</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="D19" s="5" t="s">
-        <x:v>119</x:v>
+        <x:v>93</x:v>
       </x:c>
       <x:c r="E19" s="5"/>
       <x:c r="F19" s="5" t="s">
-        <x:v>120</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="G19" s="5" t="s">
-        <x:v>121</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="H19" s="5" t="s">
-        <x:v>122</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="I19" s="5" t="s">
-        <x:v>123</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
+        <x:v>97</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="52.79999923706055" hidden="0" customHeight="1">
       <x:c r="A20" s="5">
         <x:v>19.0</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
-        <x:v>124</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C20" s="5" t="s">
-        <x:v>125</x:v>
-      </x:c>
-      <x:c r="D20" s="5" t="s">
-        <x:v>126</x:v>
-      </x:c>
-      <x:c r="E20" s="5"/>
-      <x:c r="F20" s="5" t="s">
-        <x:v>120</x:v>
-      </x:c>
-      <x:c r="G20" s="5" t="str">
+        <x:v>99</x:v>
+      </x:c>
+      <x:c r="D20" s="8" t="str">
+        <x:v>Unit 6 / Week 34</x:v>
+      </x:c>
+      <x:c r="E20" s="8" t="str"/>
+      <x:c r="F20" s="8" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="G20" s="8" t="str">
         <x:v>Unit 6 Student Handout 15: Final Research Process Reflection
 Unit 6 Student Handout 16: STARLAB Portfolio Checklist
 Unit 6 Student Handout 18: Course Feedback and Legacy Reflection</x:v>
       </x:c>
-      <x:c r="H20" s="5" t="str">
+      <x:c r="H20" s="8" t="str">
         <x:v>Unit 6 Student Handout 17: Optional Next-Step Plan
-Unit 6 Appendices O-S (optional or teacher reference)</x:v>
-      </x:c>
-      <x:c r="I20" s="5" t="s">
-        <x:v>127</x:v>
+Unit 6 Appendices O-S: optional / teacher reference</x:v>
+      </x:c>
+      <x:c r="I20" s="8" t="str">
+        <x:v>Final course closure deck. No next deck follows.</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1"/>
@@ -5161,19 +5067,19 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="s">
-        <x:v>128</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="B1" s="4" t="s">
-        <x:v>129</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="C1" s="4" t="s">
-        <x:v>130</x:v>
+        <x:v>102</x:v>
       </x:c>
       <x:c r="D1" s="4" t="s">
-        <x:v>131</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E1" s="4" t="s">
-        <x:v>132</x:v>
+        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -5181,81 +5087,81 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B2" s="5" t="s">
-        <x:v>133</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="C2" s="5" t="s">
-        <x:v>134</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="D2" s="5" t="s">
-        <x:v>135</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="E2" s="5" t="s">
-        <x:v>136</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="s">
-        <x:v>38</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
-        <x:v>137</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="C3" s="5" t="s">
-        <x:v>138</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="D3" s="5" t="s">
-        <x:v>139</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="E3" s="5" t="s">
-        <x:v>140</x:v>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="5" t="s">
-        <x:v>45</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>141</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="C4" s="5" t="s">
-        <x:v>142</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="D4" s="5" t="s">
-        <x:v>143</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="E4" s="5" t="s">
-        <x:v>144</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="5" t="s">
-        <x:v>73</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>145</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="C5" s="5" t="s">
-        <x:v>146</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="D5" s="5" t="s">
-        <x:v>147</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="E5" s="5" t="s">
-        <x:v>148</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="5" t="s">
-        <x:v>89</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>149</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="C6" s="5" t="s">
-        <x:v>150</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="D6" s="5" t="s">
-        <x:v>151</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="E6" s="5" t="str">
         <x:v>Student Handouts 1-11; Appendixes A-O and Q-S; Unit 6 Appendix L is the final oral rubric</x:v>
@@ -5263,19 +5169,19 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="5" t="s">
-        <x:v>120</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>152</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
         <x:v>Presentation, required public showcase, Q&amp;A, reflection, portfolio, and next steps</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
-        <x:v>153</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="E7" s="5" t="s">
-        <x:v>154</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1"/>
@@ -6274,10 +6180,10 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="s">
-        <x:v>155</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B1" s="4" t="s">
-        <x:v>156</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -6285,7 +6191,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B2" s="5" t="s">
-        <x:v>157</x:v>
+        <x:v>129</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6293,7 +6199,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
-        <x:v>158</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -6301,7 +6207,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>159</x:v>
+        <x:v>131</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -6309,7 +6215,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>160</x:v>
+        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6317,7 +6223,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>161</x:v>
+        <x:v>133</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -6330,18 +6236,18 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="5" t="s">
-        <x:v>162</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B8" s="5" t="s">
-        <x:v>163</x:v>
+        <x:v>135</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="5" t="s">
-        <x:v>164</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="B9" s="5" t="s">
-        <x:v>165</x:v>
+        <x:v>137</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>

<commit_message>
Align target decks with print index
</commit_message>
<xml_diff>
--- a/Teacher Resources (Start Here)/06_STARLAB_Master_Print_Packet_Index.xlsx
+++ b/Teacher Resources (Start Here)/06_STARLAB_Master_Print_Packet_Index.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R2730892ae6044289"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Packet Index" sheetId="2" r:id="R7f7fed98e2d24fc3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Print Queue" sheetId="3" r:id="Ra6dbc8079c654db8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Unit" sheetId="4" r:id="R500c174791e84cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Type Key" sheetId="5" r:id="Rcf33a24bc93742ce"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R37d9d0116a334240"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Packet Index" sheetId="2" r:id="Rb13766931e3f4f9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Print Queue" sheetId="3" r:id="R28019e65321e4255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Unit" sheetId="4" r:id="Rb8808cd605f04a7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Type Key" sheetId="5" r:id="Ra35ac0bbfa71454d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -173,9 +173,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Deck 12</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Use after initial graphs/calculations; revisit before interpretation.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Scientific Report Structure</x:t>
@@ -2103,7 +2100,7 @@
         <x:v>Teach graphing and visual ethics in Week 19; revisit the visual standards during Week 24 results writing.</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="52.79999923706055" hidden="0" customHeight="1">
+    <x:row r="13" ht="92.4000015258789" hidden="0" customHeight="1">
       <x:c r="A13" s="5">
         <x:v>12.0</x:v>
       </x:c>
@@ -2123,16 +2120,20 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="G13" s="8" t="str">
-        <x:v>Unit 4 Student Handout 11: Error, Uncertainty, and Limitations Review
+        <x:v>Week 19 required:
+Unit 4 Student Handouts 9-12
+Unit 4 Appendices H-K
+Week 20 revisit required:
 Unit 4 Student Handouts 13-17
-Unit 4 Appendices J and N</x:v>
+Unit 4 Appendix N</x:v>
       </x:c>
       <x:c r="H13" s="8" t="str">
-        <x:v>Unit 4 Appendices L-M and O-Q (teacher reference)
+        <x:v>Week 20 optional / teacher reference:
+Unit 4 Appendices L-M and O-Q
 Project-specific uncertainty examples</x:v>
       </x:c>
-      <x:c r="I13" s="8" t="s">
-        <x:v>51</x:v>
+      <x:c r="I13" s="8" t="str">
+        <x:v>Teach error, uncertainty, variability, and limitations in Week 19; revisit the relevant ideas before students finalize interpretation and claims in Week 20.</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="198" hidden="0" customHeight="1">
@@ -2140,10 +2141,10 @@
         <x:v>13.0</x:v>
       </x:c>
       <x:c r="B14" s="5" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="C14" s="5" t="s">
         <x:v>52</x:v>
-      </x:c>
-      <x:c r="C14" s="5" t="s">
-        <x:v>53</x:v>
       </x:c>
       <x:c r="D14" s="8" t="str">
         <x:v>Unit 5 / Week 21</x:v>
@@ -2152,7 +2153,7 @@
         <x:v>Unit 5 / Weeks 22, 23, and 26</x:v>
       </x:c>
       <x:c r="F14" s="8" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G14" s="8" t="str">
         <x:v>Week 21 required:
@@ -2169,7 +2170,7 @@
 Unit 5 Appendices J-L</x:v>
       </x:c>
       <x:c r="H14" s="8" t="s">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="I14" s="8" t="str">
         <x:v>Teach report architecture in Week 21; revisit the relevant report-section structure in Weeks 22, 23, and 26.</x:v>
@@ -2180,10 +2181,10 @@
         <x:v>14.0</x:v>
       </x:c>
       <x:c r="B15" s="5" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="C15" s="5" t="s">
         <x:v>56</x:v>
-      </x:c>
-      <x:c r="C15" s="5" t="s">
-        <x:v>57</x:v>
       </x:c>
       <x:c r="D15" s="8" t="str">
         <x:v>Unit 5 / Week 25</x:v>
@@ -2209,26 +2210,26 @@
         <x:v>15.0</x:v>
       </x:c>
       <x:c r="B16" s="5" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="C16" s="5" t="s">
         <x:v>58</x:v>
-      </x:c>
-      <x:c r="C16" s="5" t="s">
-        <x:v>59</x:v>
       </x:c>
       <x:c r="D16" s="8" t="str">
         <x:v>Unit 5 / Week 27</x:v>
       </x:c>
       <x:c r="E16" s="8" t="str"/>
       <x:c r="F16" s="8" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="G16" s="8" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="H16" s="8" t="s">
         <x:v>60</x:v>
       </x:c>
-      <x:c r="H16" s="8" t="s">
+      <x:c r="I16" s="8" t="s">
         <x:v>61</x:v>
-      </x:c>
-      <x:c r="I16" s="8" t="s">
-        <x:v>62</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="66" hidden="0" customHeight="1">
@@ -2236,10 +2237,10 @@
         <x:v>16.0</x:v>
       </x:c>
       <x:c r="B17" s="5" t="s">
+        <x:v>62</x:v>
+      </x:c>
+      <x:c r="C17" s="5" t="s">
         <x:v>63</x:v>
-      </x:c>
-      <x:c r="C17" s="5" t="s">
-        <x:v>64</x:v>
       </x:c>
       <x:c r="D17" s="8" t="str">
         <x:v>Unit 5 / Week 28</x:v>
@@ -2248,7 +2249,7 @@
         <x:v>Unit 6 / Week 32</x:v>
       </x:c>
       <x:c r="F17" s="8" t="s">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="G17" s="8" t="str">
         <x:v>Unit 5 Student Handout 10: Presentation Planning Guide
@@ -2261,7 +2262,7 @@
 Unit 6 Appendices I-K (teacher event references)</x:v>
       </x:c>
       <x:c r="I17" s="8" t="s">
-        <x:v>66</x:v>
+        <x:v>65</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="39.599998474121094" hidden="0" customHeight="1">
@@ -2269,10 +2270,10 @@
         <x:v>17.0</x:v>
       </x:c>
       <x:c r="B18" s="5" t="s">
+        <x:v>66</x:v>
+      </x:c>
+      <x:c r="C18" s="5" t="s">
         <x:v>67</x:v>
-      </x:c>
-      <x:c r="C18" s="5" t="s">
-        <x:v>68</x:v>
       </x:c>
       <x:c r="D18" s="8" t="str">
         <x:v>Unit 6 / Week 29</x:v>
@@ -2281,7 +2282,7 @@
         <x:v>Unit 5 / Week 28 preview; Unit 6 / Week 30 revisit</x:v>
       </x:c>
       <x:c r="F18" s="8" t="s">
-        <x:v>65</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="G18" s="8" t="str">
         <x:v>Unit 5 Student Handouts 10-11
@@ -2300,10 +2301,10 @@
         <x:v>18.0</x:v>
       </x:c>
       <x:c r="B19" s="5" t="s">
+        <x:v>68</x:v>
+      </x:c>
+      <x:c r="C19" s="5" t="s">
         <x:v>69</x:v>
-      </x:c>
-      <x:c r="C19" s="5" t="s">
-        <x:v>70</x:v>
       </x:c>
       <x:c r="D19" s="8" t="str">
         <x:v>Unit 6 / Week 31</x:v>
@@ -2312,7 +2313,7 @@
         <x:v>Unit 6 / Week 32</x:v>
       </x:c>
       <x:c r="F19" s="8" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="G19" s="8" t="str">
         <x:v>Week 31 required:
@@ -2337,17 +2338,17 @@
         <x:v>19.0</x:v>
       </x:c>
       <x:c r="B20" s="5" t="s">
+        <x:v>71</x:v>
+      </x:c>
+      <x:c r="C20" s="5" t="s">
         <x:v>72</x:v>
-      </x:c>
-      <x:c r="C20" s="5" t="s">
-        <x:v>73</x:v>
       </x:c>
       <x:c r="D20" s="8" t="str">
         <x:v>Unit 6 / Week 34</x:v>
       </x:c>
       <x:c r="E20" s="8" t="str"/>
       <x:c r="F20" s="8" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="G20" s="8" t="str">
         <x:v>Unit 6 Student Handout 15: Final Research Process Reflection
@@ -5004,19 +5005,19 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="s">
+        <x:v>73</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="s">
         <x:v>74</x:v>
       </x:c>
-      <x:c r="B1" s="4" t="s">
+      <x:c r="C1" s="4" t="s">
         <x:v>75</x:v>
       </x:c>
-      <x:c r="C1" s="4" t="s">
+      <x:c r="D1" s="4" t="s">
         <x:v>76</x:v>
       </x:c>
-      <x:c r="D1" s="4" t="s">
+      <x:c r="E1" s="4" t="s">
         <x:v>77</x:v>
-      </x:c>
-      <x:c r="E1" s="4" t="s">
-        <x:v>78</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -5024,16 +5025,16 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B2" s="5" t="s">
+        <x:v>78</x:v>
+      </x:c>
+      <x:c r="C2" s="5" t="s">
         <x:v>79</x:v>
       </x:c>
-      <x:c r="C2" s="5" t="s">
+      <x:c r="D2" s="5" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="s">
+      <x:c r="E2" s="5" t="s">
         <x:v>81</x:v>
-      </x:c>
-      <x:c r="E2" s="5" t="s">
-        <x:v>82</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -5041,16 +5042,16 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
+        <x:v>82</x:v>
+      </x:c>
+      <x:c r="C3" s="5" t="s">
         <x:v>83</x:v>
       </x:c>
-      <x:c r="C3" s="5" t="s">
+      <x:c r="D3" s="5" t="s">
         <x:v>84</x:v>
       </x:c>
-      <x:c r="D3" s="5" t="s">
+      <x:c r="E3" s="5" t="s">
         <x:v>85</x:v>
-      </x:c>
-      <x:c r="E3" s="5" t="s">
-        <x:v>86</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -5058,16 +5059,16 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
+        <x:v>86</x:v>
+      </x:c>
+      <x:c r="C4" s="5" t="s">
         <x:v>87</x:v>
       </x:c>
-      <x:c r="C4" s="5" t="s">
+      <x:c r="D4" s="5" t="s">
         <x:v>88</x:v>
       </x:c>
-      <x:c r="D4" s="5" t="s">
+      <x:c r="E4" s="5" t="s">
         <x:v>89</x:v>
-      </x:c>
-      <x:c r="E4" s="5" t="s">
-        <x:v>90</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -5075,30 +5076,30 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
+        <x:v>90</x:v>
+      </x:c>
+      <x:c r="C5" s="5" t="s">
         <x:v>91</x:v>
       </x:c>
-      <x:c r="C5" s="5" t="s">
+      <x:c r="D5" s="5" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="D5" s="5" t="s">
+      <x:c r="E5" s="5" t="s">
         <x:v>93</x:v>
-      </x:c>
-      <x:c r="E5" s="5" t="s">
-        <x:v>94</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="5" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
+        <x:v>94</x:v>
+      </x:c>
+      <x:c r="C6" s="5" t="s">
         <x:v>95</x:v>
       </x:c>
-      <x:c r="C6" s="5" t="s">
+      <x:c r="D6" s="5" t="s">
         <x:v>96</x:v>
-      </x:c>
-      <x:c r="D6" s="5" t="s">
-        <x:v>97</x:v>
       </x:c>
       <x:c r="E6" s="5" t="str">
         <x:v>Student Handouts 1-11; Appendixes A-O and Q-S; Unit 6 Appendix L is the final oral rubric</x:v>
@@ -5106,19 +5107,19 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="5" t="s">
-        <x:v>71</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B7" s="5" t="s">
-        <x:v>98</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="C7" s="5" t="str">
         <x:v>Presentation, required public showcase, Q&amp;A, reflection, portfolio, and next steps</x:v>
       </x:c>
       <x:c r="D7" s="5" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="E7" s="5" t="s">
         <x:v>99</x:v>
-      </x:c>
-      <x:c r="E7" s="5" t="s">
-        <x:v>100</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1"/>
@@ -6117,10 +6118,10 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" s="4" t="s">
+        <x:v>100</x:v>
+      </x:c>
+      <x:c r="B1" s="4" t="s">
         <x:v>101</x:v>
-      </x:c>
-      <x:c r="B1" s="4" t="s">
-        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -6128,7 +6129,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B2" s="5" t="s">
-        <x:v>103</x:v>
+        <x:v>102</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
@@ -6136,7 +6137,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B3" s="5" t="s">
-        <x:v>104</x:v>
+        <x:v>103</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -6144,7 +6145,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B4" s="5" t="s">
-        <x:v>105</x:v>
+        <x:v>104</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -6152,7 +6153,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B5" s="5" t="s">
-        <x:v>106</x:v>
+        <x:v>105</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -6160,7 +6161,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B6" s="5" t="s">
-        <x:v>107</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -6173,18 +6174,18 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="5" t="s">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
         <x:v>108</x:v>
-      </x:c>
-      <x:c r="B8" s="5" t="s">
-        <x:v>109</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="5" t="s">
+        <x:v>109</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="s">
         <x:v>110</x:v>
-      </x:c>
-      <x:c r="B9" s="5" t="s">
-        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>

<commit_message>
Validate first-month print packets
</commit_message>
<xml_diff>
--- a/Teacher Resources (Start Here)/06_STARLAB_Master_Print_Packet_Index.xlsx
+++ b/Teacher Resources (Start Here)/06_STARLAB_Master_Print_Packet_Index.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="Rc75939a0b50f4161"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Packet Index" sheetId="2" r:id="Ra6aee84c7ee744ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Print Queue" sheetId="3" r:id="Rffd4691c09f041ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Unit" sheetId="4" r:id="R1bb651d7f797403d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Type Key" sheetId="5" r:id="R7efaf8d206594452"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R4546ef5cb1334b10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Print Packet Index" sheetId="2" r:id="R7410611f7bc04cdf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quick Print Queue" sheetId="3" r:id="R4b761042eeae4ab1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="By Unit" sheetId="4" r:id="R2db690687d6f42a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resource Type Key" sheetId="5" r:id="R50b6e8cc0b024e72"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -334,9 +334,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">The unit folder(s) where the required handouts/appendixes live.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Materials students should have for the lesson or lesson sequence.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">H</x:t>
@@ -658,7 +655,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="3" t="str">
-        <x:v>This spreadsheet separates required student copies from optional or teacher-reference materials and distinguishes primary teaching moments from later revisit use.</x:v>
+        <x:v>This spreadsheet separates required print materials from optional or teacher-reference materials and distinguishes primary teaching moments from later revisit use.</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
@@ -1769,12 +1766,9 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="G3" s="8" t="str">
-        <x:v>Unit 1 Student Handout 3: Research Interest Inventory
-Unit 1 Student Handout 6: From Topic to Research Question
-Unit 1 Student Handout 7: Question Quality Test
-Unit 1 Student Handout 8: Preliminary Project Pitch
-Unit 1 Appendix E: Strong vs. Weak Research Questions
-Unit 1 Appendix G: Engineering Design Problem Guide</x:v>
+        <x:v>Week 2 required packet (shared with Deck 4):
+Unit 1 Student Handouts 5-8
+Unit 1 Appendices D-H</x:v>
       </x:c>
       <x:c r="H3" s="8" t="str">
         <x:v>Unit 1 Appendix I: Optional Project Card Sorting Activity
@@ -1846,10 +1840,9 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="G5" s="8" t="str">
-        <x:v>Week 2 required:
-Unit 1 Student Handout 5: Experimental Design Practice
-Unit 1 Appendix D: Experimental Design Vocabulary
-Unit 1 Appendix G: Engineering Design Problem Guide
+        <x:v>Week 2 required packet (shared with Deck 2):
+Unit 1 Student Handouts 5-8
+Unit 1 Appendices D-H
 Week 3 revisit required:
 Unit 2 Student Handout 3: Hypothesis and Design Criteria Builder
 Unit 2 Student Handout 4: Variables, Controls, Criteria, and Constraints Organizer
@@ -3387,7 +3380,7 @@
         <x:v>Deck Use</x:v>
       </x:c>
       <x:c r="D1" s="6" t="str">
-        <x:v>Required Student Copies</x:v>
+        <x:v>Required Print Materials</x:v>
       </x:c>
       <x:c r="E1" s="6" t="str">
         <x:v>Optional / Teacher Reference</x:v>
@@ -6187,8 +6180,8 @@
       <x:c r="A6" s="5" t="s">
         <x:v>12</x:v>
       </x:c>
-      <x:c r="B6" s="5" t="s">
-        <x:v>104</x:v>
+      <x:c r="B6" s="5" t="str">
+        <x:v>Materials that must be available for the lesson or lesson sequence. This may include student copies and required teacher references.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -6201,18 +6194,18 @@
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="5" t="s">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="B8" s="5" t="s">
         <x:v>105</x:v>
-      </x:c>
-      <x:c r="B8" s="5" t="s">
-        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="5" t="s">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="B9" s="5" t="s">
         <x:v>107</x:v>
-      </x:c>
-      <x:c r="B9" s="5" t="s">
-        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>